<commit_message>
Deploying to gh-pages from  @ e4cb09a77d0e89dde14083e3663f06d49053d314 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2026_8-1-1.xlsx
+++ b/assets/excel/2026_8-1-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BiesterChristophLSN\Desktop\MZ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B105DCE-8A5D-44E7-8AE5-D5214D9A890E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BE276B5-8110-4F1C-A635-6AF0D4246654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{D43F1882-7F0B-4535-9074-3F9134A0911D}"/>
+    <workbookView xWindow="20052" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D43F1882-7F0B-4535-9074-3F9134A0911D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="25">
   <si>
     <t>Migration und Teilhabe in Niedersachsen - Integrationsmonitoring 2026</t>
   </si>
@@ -88,19 +88,10 @@
     <t>65 und älter</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Hochrechnung anhand der Bevölkerungsfortschreibung auf Basis des Zensus 2011. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe. Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren. </t>
-  </si>
-  <si>
-    <t>2) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes</t>
-  </si>
-  <si>
     <t>https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Bevoelkerung/Haushalte-Familien/Methoden/mikrozensus-2020.html</t>
   </si>
   <si>
     <t>Quelle: Mikrozensus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Niedersächsisches Ministerium für Soziales, Gesundheit und Gleichstellung (Hrsg.), </t>
   </si>
   <si>
     <t>Vervielfältigung und Verbreitung, auch auszugsweise, mit Quellenangabe gestattet.</t>
@@ -109,7 +100,19 @@
     <t>https://www.integrationsmonitoring.niedersachsen.de</t>
   </si>
   <si>
-    <t xml:space="preserve">© Landesamt für Statistik Niedersachsen, Hannover 2026,                                                               </t>
+    <t>1)  Ab der Veröffentlichung der Endergebnisse 2023 und der Erstergebnisse 2024 werden für die Hochrechnung des Mikrozensus Daten der Bevölkerungsfortschreibung herangezogen, die auf den Eckwerten des Zensus 2022 basieren. Die Hochrechnung für die Jahre vor 2011 sowie für bislang veröffentlichte Ergebnisse des Mikrozensus 2011-2013 basiert auf den fortgeschriebenen Ergebnissen der Volkszählung 1987. In 2016 erfolgte die Umstellung auf eine neue Mikrozensus-Stichprobe (auf Basis des Zensus 2011). Ab 2017 wird nur noch die Bevölkerung in Privathaushalten (ohne Gemeinschaftsunterkünfte) ausgewiesen. Dadurch ergibt sich jeweils eine eingeschränkte Vergleichbarkeit mit den Vorjahren.</t>
+  </si>
+  <si>
+    <t>2) Seit dem Jahr 2018 wird im Mikrozensus der Migrationshintergrund im weiteren Sinne jährlich berichtet. Die in der Tabelle ab dem Jahr 2018 abgebildeten Daten zum Migrationshintergrund entsprechen dem Migrationshintergrund im weiteren Sinne, bis 2017 wird der Migrationshintergrund im engeren Sinne abgebildet. Die Vergleichbarkeit ist dadurch eingeschränkt.</t>
+  </si>
+  <si>
+    <t>3) Die Ergebnisse des Mikrozensus 2020 sind unter anderem aufgrund methodischer Effekte im Rahmen einer Neugestaltung der Erhebung sowie insbesondere aufgrund der Folgen der Corona-Pandemie in Ihrer Datenqualität eingeschränkt. Auf die Verwendung dieser Ergebnisse wird daher verzichtet. Weitere Informationen zur methodischen Neugestaltung des Mikrozensus ab 2020 und zu den Auswirkungen der Neugestaltung und der Corona-Krise auf die Ergebnisse des Jahres 2020 finden Sie auf der Informationsseite des Statistischen Bundesamtes:</t>
+  </si>
+  <si>
+    <t>Niedersächsisches Ministerium für Soziales, Gesundheit und Gleichstellung (Hrsg.),</t>
+  </si>
+  <si>
+    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,</t>
   </si>
 </sst>
 </file>
@@ -339,12 +342,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -405,9 +409,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -429,6 +430,30 @@
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -447,59 +472,47 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
+    <cellStyle name="Link" xfId="3" builtinId="8"/>
     <cellStyle name="Link 2" xfId="2" xr:uid="{67F61250-2934-47B0-AE00-BF52AD7977C6}"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard_Tabelle_A_6_HT" xfId="1" xr:uid="{782C9885-669D-485A-ACDF-066880B73A8E}"/>
@@ -518,9 +531,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -558,7 +571,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -664,7 +677,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -806,7 +819,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -815,15 +828,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E78AA4F0-A99B-4EA6-A04C-A350B1A3D9D9}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="B1:L215"/>
+  <dimension ref="B1:M215"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="22" customWidth="1"/>
-    <col min="2" max="16384" width="11.42578125" style="22"/>
+    <col min="1" max="1" width="5.7109375" style="21" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="21"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="28" t="s">
         <v>0</v>
       </c>
     </row>
@@ -843,7 +856,7 @@
       <c r="K3" s="3"/>
     </row>
     <row r="4" spans="2:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="29" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1"/>
@@ -857,29 +870,29 @@
       <c r="K4" s="4"/>
     </row>
     <row r="5" spans="2:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="2:12" s="45" customFormat="1" ht="8.25" x14ac:dyDescent="0.25">
-      <c r="B6" s="29" t="s">
+    <row r="6" spans="2:12" s="30" customFormat="1" ht="8.25" x14ac:dyDescent="0.25">
+      <c r="B6" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="D6" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="35"/>
+      <c r="E6" s="43"/>
       <c r="F6" s="44"/>
-      <c r="G6" s="37" t="s">
+      <c r="G6" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
+      <c r="H6" s="46"/>
+      <c r="I6" s="46"/>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
     </row>
-    <row r="7" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="30"/>
-      <c r="C7" s="33"/>
+    <row r="7" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="37"/>
+      <c r="C7" s="40"/>
       <c r="D7" s="9" t="s">
         <v>7</v>
       </c>
@@ -901,23 +914,23 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="31"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="41" t="s">
+    <row r="8" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="38"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="42"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="37" t="s">
+      <c r="E8" s="48"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="46"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
     </row>
-    <row r="9" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12">
         <v>1</v>
       </c>
@@ -946,1981 +959,1981 @@
       <c r="K9" s="12"/>
       <c r="L9" s="12"/>
     </row>
-    <row r="10" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="23" t="s">
+    <row r="10" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="23">
+      <c r="C10" s="22">
         <v>2025</v>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="23">
         <v>59.9</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="23">
         <v>55.1</v>
       </c>
-      <c r="F10" s="24">
+      <c r="F10" s="23">
         <v>114.9</v>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="24">
         <v>24.599589322381927</v>
       </c>
-      <c r="H10" s="25">
+      <c r="H10" s="24">
         <v>31.04225352112676</v>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="24">
         <v>24.138655462184875</v>
       </c>
       <c r="J10" s="12"/>
       <c r="K10" s="12"/>
       <c r="L10" s="12"/>
     </row>
-    <row r="11" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="23" t="s">
+    <row r="11" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="23">
+      <c r="C11" s="22">
         <v>2025</v>
       </c>
-      <c r="D11" s="24">
+      <c r="D11" s="23">
         <v>151.1</v>
       </c>
-      <c r="E11" s="24">
+      <c r="E11" s="23">
         <v>152.4</v>
       </c>
-      <c r="F11" s="24">
+      <c r="F11" s="23">
         <v>303.5</v>
       </c>
-      <c r="G11" s="25">
+      <c r="G11" s="24">
         <v>18.615251940372058</v>
       </c>
-      <c r="H11" s="25">
+      <c r="H11" s="24">
         <v>23.775351014040563</v>
       </c>
-      <c r="I11" s="25">
+      <c r="I11" s="24">
         <v>18.907301270869674</v>
       </c>
       <c r="J11" s="12"/>
       <c r="K11" s="12"/>
       <c r="L11" s="12"/>
     </row>
-    <row r="12" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="23" t="s">
+    <row r="12" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="23">
+      <c r="C12" s="22">
         <v>2025</v>
       </c>
-      <c r="D12" s="24">
+      <c r="D12" s="23">
         <v>131.1</v>
       </c>
-      <c r="E12" s="24">
+      <c r="E12" s="23">
         <v>144.69999999999999</v>
       </c>
-      <c r="F12" s="24">
+      <c r="F12" s="23">
         <v>275.8</v>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="24">
         <v>13.11</v>
       </c>
-      <c r="H12" s="25">
+      <c r="H12" s="24">
         <v>16.411477826925257</v>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="24">
         <v>13.610343466245558</v>
       </c>
       <c r="J12" s="12"/>
       <c r="K12" s="12"/>
       <c r="L12" s="12"/>
     </row>
-    <row r="13" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="23" t="s">
+    <row r="13" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="23">
+      <c r="C13" s="22">
         <v>2025</v>
       </c>
-      <c r="D13" s="24">
+      <c r="D13" s="23">
         <v>74.900000000000006</v>
       </c>
-      <c r="E13" s="24">
+      <c r="E13" s="23">
         <v>88.4</v>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="23">
         <v>163.30000000000001</v>
       </c>
-      <c r="G13" s="25">
+      <c r="G13" s="24">
         <v>9.6970481615743154</v>
       </c>
-      <c r="H13" s="25">
+      <c r="H13" s="24">
         <v>10.473933649289101</v>
       </c>
-      <c r="I13" s="25">
+      <c r="I13" s="24">
         <v>9.5788362271234178</v>
       </c>
       <c r="J13" s="12"/>
       <c r="K13" s="12"/>
       <c r="L13" s="12"/>
     </row>
-    <row r="14" spans="2:12" s="45" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="50" t="s">
+    <row r="14" spans="2:12" s="30" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="25">
         <v>2025</v>
       </c>
-      <c r="D14" s="27">
+      <c r="D14" s="26">
         <v>417</v>
       </c>
-      <c r="E14" s="27">
+      <c r="E14" s="26">
         <v>440.6</v>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="26">
         <v>857.6</v>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="26">
         <v>14.747489036638846</v>
       </c>
-      <c r="H14" s="27">
+      <c r="H14" s="26">
         <v>17.317820926027832</v>
       </c>
-      <c r="I14" s="27">
+      <c r="I14" s="26">
         <v>14.754662445805518</v>
       </c>
       <c r="J14" s="12"/>
       <c r="K14" s="12"/>
       <c r="L14" s="12"/>
     </row>
-    <row r="15" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="23" t="s">
+    <row r="15" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="23">
+      <c r="C15" s="22">
         <v>2024</v>
       </c>
-      <c r="D15" s="24">
+      <c r="D15" s="23">
         <v>57.4</v>
       </c>
-      <c r="E15" s="24">
+      <c r="E15" s="23">
         <v>52.8</v>
       </c>
-      <c r="F15" s="24">
+      <c r="F15" s="23">
         <v>110.3</v>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="24">
         <v>22.96</v>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="24">
         <v>27.862796833773086</v>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="24">
         <v>22.405037578712168</v>
       </c>
       <c r="J15" s="12"/>
       <c r="K15" s="12"/>
       <c r="L15" s="12"/>
     </row>
-    <row r="16" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="23" t="s">
+    <row r="16" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="23">
+      <c r="C16" s="22">
         <v>2024</v>
       </c>
-      <c r="D16" s="24">
+      <c r="D16" s="23">
         <v>145</v>
       </c>
-      <c r="E16" s="24">
+      <c r="E16" s="23">
         <v>151.80000000000001</v>
       </c>
-      <c r="F16" s="24">
+      <c r="F16" s="23">
         <v>296.8</v>
       </c>
-      <c r="G16" s="25">
+      <c r="G16" s="24">
         <v>17.894606935702829</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="24">
         <v>23.781920726930913</v>
       </c>
-      <c r="I16" s="25">
+      <c r="I16" s="24">
         <v>18.546522527026184</v>
       </c>
       <c r="J16" s="12"/>
       <c r="K16" s="12"/>
       <c r="L16" s="12"/>
     </row>
-    <row r="17" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="23" t="s">
+    <row r="17" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="23">
+      <c r="C17" s="22">
         <v>2024</v>
       </c>
-      <c r="D17" s="24">
+      <c r="D17" s="23">
         <v>125.7</v>
       </c>
-      <c r="E17" s="24">
+      <c r="E17" s="23">
         <v>144.80000000000001</v>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="23">
         <v>270.5</v>
       </c>
-      <c r="G17" s="25">
+      <c r="G17" s="24">
         <v>12.477665276950567</v>
       </c>
-      <c r="H17" s="25">
+      <c r="H17" s="24">
         <v>16.191434641619146</v>
       </c>
-      <c r="I17" s="25">
+      <c r="I17" s="24">
         <v>13.217042900420209</v>
       </c>
       <c r="J17" s="12"/>
       <c r="K17" s="12"/>
       <c r="L17" s="12"/>
     </row>
-    <row r="18" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="23" t="s">
+    <row r="18" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="23">
+      <c r="C18" s="22">
         <v>2024</v>
       </c>
-      <c r="D18" s="24">
+      <c r="D18" s="23">
         <v>74.2</v>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="23">
         <v>89.9</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="23">
         <v>164.1</v>
       </c>
-      <c r="G18" s="25">
+      <c r="G18" s="24">
         <v>9.6803652968036538</v>
       </c>
-      <c r="H18" s="25">
+      <c r="H18" s="24">
         <v>10.805288461538462</v>
       </c>
-      <c r="I18" s="25">
+      <c r="I18" s="24">
         <v>9.7192608386638231</v>
       </c>
       <c r="J18" s="12"/>
       <c r="K18" s="12"/>
       <c r="L18" s="12"/>
     </row>
-    <row r="19" spans="2:12" s="45" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="26" t="s">
+    <row r="19" spans="2:12" s="30" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="26">
+      <c r="C19" s="25">
         <v>2024</v>
       </c>
-      <c r="D19" s="26">
+      <c r="D19" s="25">
         <v>402.3</v>
       </c>
-      <c r="E19" s="27">
+      <c r="E19" s="26">
         <v>439.4</v>
       </c>
-      <c r="F19" s="26">
+      <c r="F19" s="25">
         <v>841.7</v>
       </c>
-      <c r="G19" s="27">
+      <c r="G19" s="26">
         <v>14.194481687954275</v>
       </c>
-      <c r="H19" s="27">
+      <c r="H19" s="26">
         <v>17.2043852779953</v>
       </c>
-      <c r="I19" s="27">
+      <c r="I19" s="26">
         <v>14.443338595648294</v>
       </c>
       <c r="J19" s="12"/>
       <c r="K19" s="12"/>
       <c r="L19" s="12"/>
     </row>
-    <row r="20" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="23" t="s">
+    <row r="20" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="23">
+      <c r="C20" s="22">
         <v>2023</v>
       </c>
-      <c r="D20" s="24">
+      <c r="D20" s="23">
         <v>50.4</v>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="23">
         <v>50.2</v>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="23">
         <v>100.6</v>
       </c>
-      <c r="G20" s="25">
+      <c r="G20" s="24">
         <v>19.881656804733726</v>
       </c>
-      <c r="H20" s="25">
+      <c r="H20" s="24">
         <v>24.87611496531219</v>
       </c>
-      <c r="I20" s="25">
+      <c r="I20" s="24">
         <v>19.897151898734176</v>
       </c>
       <c r="J20" s="12"/>
       <c r="K20" s="12"/>
       <c r="L20" s="12"/>
     </row>
-    <row r="21" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="23" t="s">
+    <row r="21" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="23">
+      <c r="C21" s="22">
         <v>2023</v>
       </c>
-      <c r="D21" s="24">
+      <c r="D21" s="23">
         <v>136.69999999999999</v>
       </c>
-      <c r="E21" s="24">
+      <c r="E21" s="23">
         <v>136.5</v>
       </c>
-      <c r="F21" s="24">
+      <c r="F21" s="23">
         <v>273.2</v>
       </c>
-      <c r="G21" s="25">
+      <c r="G21" s="24">
         <v>16.964507321916109</v>
       </c>
-      <c r="H21" s="25">
+      <c r="H21" s="24">
         <v>21.045328399629973</v>
       </c>
-      <c r="I21" s="25">
+      <c r="I21" s="24">
         <v>17.172669558111757</v>
       </c>
       <c r="J21" s="12"/>
       <c r="K21" s="12"/>
       <c r="L21" s="12"/>
     </row>
-    <row r="22" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="23" t="s">
+    <row r="22" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="23">
+      <c r="C22" s="22">
         <v>2023</v>
       </c>
-      <c r="D22" s="24">
+      <c r="D22" s="23">
         <v>115.9</v>
       </c>
-      <c r="E22" s="24">
+      <c r="E22" s="23">
         <v>127.5</v>
       </c>
-      <c r="F22" s="24">
+      <c r="F22" s="23">
         <v>243.4</v>
       </c>
-      <c r="G22" s="25">
+      <c r="G22" s="24">
         <v>11.289694135982858</v>
       </c>
-      <c r="H22" s="25">
+      <c r="H22" s="24">
         <v>13.668524871355062</v>
       </c>
-      <c r="I22" s="25">
+      <c r="I22" s="24">
         <v>11.663232545881451</v>
       </c>
       <c r="J22" s="12"/>
       <c r="K22" s="12"/>
       <c r="L22" s="12"/>
     </row>
-    <row r="23" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="23" t="s">
+    <row r="23" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="23">
+      <c r="C23" s="22">
         <v>2023</v>
       </c>
-      <c r="D23" s="24">
+      <c r="D23" s="23">
         <v>62.2</v>
       </c>
-      <c r="E23" s="24">
+      <c r="E23" s="23">
         <v>79.599999999999994</v>
       </c>
-      <c r="F23" s="24">
+      <c r="F23" s="23">
         <v>141.9</v>
       </c>
-      <c r="G23" s="25">
+      <c r="G23" s="24">
         <v>8.242777630532732</v>
       </c>
-      <c r="H23" s="25">
+      <c r="H23" s="24">
         <v>9.6088845968131338</v>
       </c>
-      <c r="I23" s="25">
+      <c r="I23" s="24">
         <v>8.5343116617549768</v>
       </c>
       <c r="J23" s="12"/>
       <c r="K23" s="12"/>
       <c r="L23" s="12"/>
     </row>
-    <row r="24" spans="2:12" s="45" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="26" t="s">
+    <row r="24" spans="2:12" s="30" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C24" s="26">
+      <c r="C24" s="25">
         <v>2023</v>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="25">
         <v>365.2</v>
       </c>
-      <c r="E24" s="27">
+      <c r="E24" s="26">
         <v>393.8</v>
       </c>
-      <c r="F24" s="26">
+      <c r="F24" s="25">
         <v>759</v>
       </c>
-      <c r="G24" s="27">
+      <c r="G24" s="26">
         <v>12.856891392360501</v>
       </c>
-      <c r="H24" s="27">
+      <c r="H24" s="26">
         <v>15.078301489451318</v>
       </c>
-      <c r="I24" s="27">
+      <c r="I24" s="26">
         <v>12.983014317237132</v>
       </c>
       <c r="J24" s="12"/>
       <c r="K24" s="12"/>
       <c r="L24" s="12"/>
     </row>
-    <row r="25" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="23" t="s">
+    <row r="25" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C25" s="23">
+      <c r="C25" s="22">
         <v>2022</v>
       </c>
-      <c r="D25" s="24">
+      <c r="D25" s="23">
         <v>51.4</v>
       </c>
-      <c r="E25" s="24">
+      <c r="E25" s="23">
         <v>50.3</v>
       </c>
-      <c r="F25" s="24">
+      <c r="F25" s="23">
         <v>101.7</v>
       </c>
-      <c r="G25" s="25">
+      <c r="G25" s="24">
         <v>19.001848428835487</v>
       </c>
-      <c r="H25" s="25">
+      <c r="H25" s="24">
         <v>23.37360594795539</v>
       </c>
-      <c r="I25" s="25">
+      <c r="I25" s="24">
         <v>18.973880597014926</v>
       </c>
       <c r="J25" s="12"/>
       <c r="K25" s="12"/>
       <c r="L25" s="12"/>
     </row>
-    <row r="26" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="23" t="s">
+    <row r="26" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="23">
+      <c r="C26" s="22">
         <v>2022</v>
       </c>
-      <c r="D26" s="24">
+      <c r="D26" s="23">
         <v>137</v>
       </c>
-      <c r="E26" s="24">
+      <c r="E26" s="23">
         <v>140.4</v>
       </c>
-      <c r="F26" s="24">
+      <c r="F26" s="23">
         <v>277.39999999999998</v>
       </c>
-      <c r="G26" s="25">
+      <c r="G26" s="24">
         <v>17.012293555196823</v>
       </c>
-      <c r="H26" s="25">
+      <c r="H26" s="24">
         <v>21.626617375231053</v>
       </c>
-      <c r="I26" s="25">
+      <c r="I26" s="24">
         <v>17.392939996238006</v>
       </c>
       <c r="J26" s="12"/>
       <c r="K26" s="12"/>
       <c r="L26" s="12"/>
     </row>
-    <row r="27" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="23" t="s">
+    <row r="27" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="22">
         <v>2022</v>
       </c>
-      <c r="D27" s="24">
+      <c r="D27" s="23">
         <v>124.3</v>
       </c>
-      <c r="E27" s="24">
+      <c r="E27" s="23">
         <v>129.80000000000001</v>
       </c>
-      <c r="F27" s="24">
+      <c r="F27" s="23">
         <v>254.1</v>
       </c>
-      <c r="G27" s="25">
+      <c r="G27" s="24">
         <v>11.856161770316671</v>
       </c>
-      <c r="H27" s="25">
+      <c r="H27" s="24">
         <v>13.614432557163836</v>
       </c>
-      <c r="I27" s="25">
+      <c r="I27" s="24">
         <v>11.920623006192532</v>
       </c>
       <c r="J27" s="12"/>
       <c r="K27" s="12"/>
       <c r="L27" s="12"/>
     </row>
-    <row r="28" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="23" t="s">
+    <row r="28" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="23">
+      <c r="C28" s="22">
         <v>2022</v>
       </c>
-      <c r="D28" s="24">
+      <c r="D28" s="23">
         <v>62.2</v>
       </c>
-      <c r="E28" s="24">
+      <c r="E28" s="23">
         <v>72.7</v>
       </c>
-      <c r="F28" s="24">
+      <c r="F28" s="23">
         <v>135</v>
       </c>
-      <c r="G28" s="25">
+      <c r="G28" s="24">
         <v>8.3010810089416793</v>
       </c>
-      <c r="H28" s="25">
+      <c r="H28" s="24">
         <v>8.7306352828149389</v>
       </c>
-      <c r="I28" s="25">
+      <c r="I28" s="24">
         <v>8.1585785943071247</v>
       </c>
       <c r="J28" s="12"/>
       <c r="K28" s="12"/>
       <c r="L28" s="12"/>
     </row>
-    <row r="29" spans="2:12" s="45" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="26" t="s">
+    <row r="29" spans="2:12" s="30" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C29" s="26">
+      <c r="C29" s="25">
         <v>2022</v>
       </c>
-      <c r="D29" s="26">
+      <c r="D29" s="25">
         <v>374.9</v>
       </c>
-      <c r="E29" s="26">
+      <c r="E29" s="25">
         <v>393.2</v>
       </c>
-      <c r="F29" s="26">
+      <c r="F29" s="25">
         <v>768.1</v>
       </c>
-      <c r="G29" s="27">
+      <c r="G29" s="26">
         <v>13.046807029754653</v>
       </c>
-      <c r="H29" s="27">
+      <c r="H29" s="26">
         <v>14.834377122161021</v>
       </c>
-      <c r="I29" s="27">
+      <c r="I29" s="26">
         <v>12.980801730548233</v>
       </c>
       <c r="J29" s="12"/>
       <c r="K29" s="12"/>
       <c r="L29" s="12"/>
     </row>
-    <row r="30" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="23" t="s">
+    <row r="30" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C30" s="23">
+      <c r="C30" s="22">
         <v>2021</v>
       </c>
-      <c r="D30" s="24">
+      <c r="D30" s="23">
         <v>56.3</v>
       </c>
-      <c r="E30" s="24">
+      <c r="E30" s="23">
         <v>51.8</v>
       </c>
-      <c r="F30" s="24">
+      <c r="F30" s="23">
         <v>108.1</v>
       </c>
-      <c r="G30" s="25">
+      <c r="G30" s="24">
         <v>17.70440251572327</v>
       </c>
-      <c r="H30" s="25">
+      <c r="H30" s="24">
         <v>17.278185456971311</v>
       </c>
-      <c r="I30" s="25">
+      <c r="I30" s="24">
         <v>17.4975720297831</v>
       </c>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
     </row>
-    <row r="31" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="23" t="s">
+    <row r="31" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C31" s="23">
+      <c r="C31" s="22">
         <v>2021</v>
       </c>
-      <c r="D31" s="24">
+      <c r="D31" s="23">
         <v>140.69999999999999</v>
       </c>
-      <c r="E31" s="24">
+      <c r="E31" s="23">
         <v>141.19999999999999</v>
       </c>
-      <c r="F31" s="24">
+      <c r="F31" s="23">
         <v>281.89999999999998</v>
       </c>
-      <c r="G31" s="25">
+      <c r="G31" s="24">
         <v>14.466378778531769</v>
       </c>
-      <c r="H31" s="25">
+      <c r="H31" s="24">
         <v>15.204048670184125</v>
       </c>
-      <c r="I31" s="25">
+      <c r="I31" s="24">
         <v>14.826697522747592</v>
       </c>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="2:12" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="23" t="s">
+    <row r="32" spans="2:12" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="23">
+      <c r="C32" s="22">
         <v>2021</v>
       </c>
-      <c r="D32" s="24">
+      <c r="D32" s="23">
         <v>124.1</v>
       </c>
-      <c r="E32" s="24">
+      <c r="E32" s="23">
         <v>131.9</v>
       </c>
-      <c r="F32" s="24">
+      <c r="F32" s="23">
         <v>256.10000000000002</v>
       </c>
-      <c r="G32" s="25">
+      <c r="G32" s="24">
         <v>10.625</v>
       </c>
-      <c r="H32" s="25">
+      <c r="H32" s="24">
         <v>11.136440391759541</v>
       </c>
-      <c r="I32" s="25">
+      <c r="I32" s="24">
         <v>10.886753953409285</v>
       </c>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
     </row>
-    <row r="33" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="23" t="s">
+    <row r="33" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C33" s="23">
+      <c r="C33" s="22">
         <v>2021</v>
       </c>
-      <c r="D33" s="24">
+      <c r="D33" s="23">
         <v>61.6</v>
       </c>
-      <c r="E33" s="24">
+      <c r="E33" s="23">
         <v>72.7</v>
       </c>
-      <c r="F33" s="24">
+      <c r="F33" s="23">
         <v>134.30000000000001</v>
       </c>
-      <c r="G33" s="25">
+      <c r="G33" s="24">
         <v>8.0250130276185505</v>
       </c>
-      <c r="H33" s="25">
+      <c r="H33" s="24">
         <v>7.870520731839342</v>
       </c>
-      <c r="I33" s="25">
+      <c r="I33" s="24">
         <v>7.9406373795305392</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
     </row>
-    <row r="34" spans="2:11" s="46" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="26" t="s">
+    <row r="34" spans="2:11" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C34" s="26">
+      <c r="C34" s="25">
         <v>2021</v>
       </c>
-      <c r="D34" s="26">
+      <c r="D34" s="25">
         <v>382.7</v>
       </c>
-      <c r="E34" s="26">
+      <c r="E34" s="25">
         <v>397.6</v>
       </c>
-      <c r="F34" s="26">
+      <c r="F34" s="25">
         <v>780.4</v>
       </c>
-      <c r="G34" s="27">
+      <c r="G34" s="26">
         <v>11.861885131574867</v>
       </c>
-      <c r="H34" s="27">
+      <c r="H34" s="26">
         <v>11.917036326579547</v>
       </c>
-      <c r="I34" s="27">
+      <c r="I34" s="26">
         <v>11.891447117802125</v>
       </c>
       <c r="J34" s="13"/>
       <c r="K34" s="13"/>
     </row>
-    <row r="35" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="23" t="s">
+    <row r="35" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C35" s="23">
+      <c r="C35" s="22">
         <v>2019</v>
       </c>
-      <c r="D35" s="24">
+      <c r="D35" s="23">
         <v>45.657209999999999</v>
       </c>
-      <c r="E35" s="24">
+      <c r="E35" s="23">
         <v>47.936019999999999</v>
       </c>
-      <c r="F35" s="24">
+      <c r="F35" s="23">
         <v>93.593230000000005</v>
       </c>
-      <c r="G35" s="25">
+      <c r="G35" s="24">
         <v>16.744907252997706</v>
       </c>
-      <c r="H35" s="25">
+      <c r="H35" s="24">
         <v>18.049068776728038</v>
       </c>
-      <c r="I35" s="25">
+      <c r="I35" s="24">
         <v>17.388415519852394</v>
       </c>
       <c r="J35" s="7"/>
       <c r="K35" s="7"/>
     </row>
-    <row r="36" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="23" t="s">
+    <row r="36" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C36" s="23">
+      <c r="C36" s="22">
         <v>2019</v>
       </c>
-      <c r="D36" s="24">
+      <c r="D36" s="23">
         <v>137.26588000000001</v>
       </c>
-      <c r="E36" s="24">
+      <c r="E36" s="23">
         <v>128.84900999999999</v>
       </c>
-      <c r="F36" s="24">
+      <c r="F36" s="23">
         <v>266.11489</v>
       </c>
-      <c r="G36" s="25">
+      <c r="G36" s="24">
         <v>17.006233497576577</v>
       </c>
-      <c r="H36" s="25">
+      <c r="H36" s="24">
         <v>16.473065850963444</v>
       </c>
-      <c r="I36" s="25">
+      <c r="I36" s="24">
         <v>16.743838060243601</v>
       </c>
       <c r="J36" s="7"/>
       <c r="K36" s="7"/>
     </row>
-    <row r="37" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="23" t="s">
+    <row r="37" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C37" s="23">
+      <c r="C37" s="22">
         <v>2019</v>
       </c>
-      <c r="D37" s="24">
+      <c r="D37" s="23">
         <v>107.7658</v>
       </c>
-      <c r="E37" s="24">
+      <c r="E37" s="23">
         <v>115.80685000000001</v>
       </c>
-      <c r="F37" s="24">
+      <c r="F37" s="23">
         <v>223.57265000000001</v>
       </c>
-      <c r="G37" s="25">
+      <c r="G37" s="24">
         <v>9.8662317726120019</v>
       </c>
-      <c r="H37" s="25">
+      <c r="H37" s="24">
         <v>10.373193698698781</v>
       </c>
-      <c r="I37" s="25">
+      <c r="I37" s="24">
         <v>10.122482717074153</v>
       </c>
       <c r="J37" s="7"/>
       <c r="K37" s="7"/>
     </row>
-    <row r="38" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="23" t="s">
+    <row r="38" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="23">
+      <c r="C38" s="22">
         <v>2019</v>
       </c>
-      <c r="D38" s="24">
+      <c r="D38" s="23">
         <v>44.276629999999997</v>
       </c>
-      <c r="E38" s="24">
+      <c r="E38" s="23">
         <v>56.083379999999998</v>
       </c>
-      <c r="F38" s="24">
+      <c r="F38" s="23">
         <v>100.36000999999999</v>
       </c>
-      <c r="G38" s="25">
+      <c r="G38" s="24">
         <v>6.1769622035587552</v>
       </c>
-      <c r="H38" s="25">
+      <c r="H38" s="24">
         <v>6.4387895782163893</v>
       </c>
-      <c r="I38" s="25">
+      <c r="I38" s="24">
         <v>6.3205911588617578</v>
       </c>
       <c r="J38" s="7"/>
       <c r="K38" s="7"/>
     </row>
-    <row r="39" spans="2:11" s="46" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="26" t="s">
+    <row r="39" spans="2:11" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C39" s="26">
+      <c r="C39" s="25">
         <v>2019</v>
       </c>
-      <c r="D39" s="28">
+      <c r="D39" s="27">
         <v>334.96552000000003</v>
       </c>
-      <c r="E39" s="28">
+      <c r="E39" s="27">
         <v>348.67526000000004</v>
       </c>
-      <c r="F39" s="28">
+      <c r="F39" s="27">
         <v>683.64078000000006</v>
       </c>
-      <c r="G39" s="27">
+      <c r="G39" s="26">
         <v>11.594974270717092</v>
       </c>
-      <c r="H39" s="27">
+      <c r="H39" s="26">
         <v>11.487735548811754</v>
       </c>
-      <c r="I39" s="27">
+      <c r="I39" s="26">
         <v>11.540030642557959</v>
       </c>
       <c r="J39" s="13"/>
       <c r="K39" s="13"/>
     </row>
-    <row r="40" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="23" t="s">
+    <row r="40" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C40" s="23">
+      <c r="C40" s="22">
         <v>2018</v>
       </c>
-      <c r="D40" s="24">
+      <c r="D40" s="23">
         <v>47.080760000000005</v>
       </c>
-      <c r="E40" s="24">
+      <c r="E40" s="23">
         <v>42.174160000000001</v>
       </c>
-      <c r="F40" s="24">
+      <c r="F40" s="23">
         <v>89.254919999999998</v>
       </c>
-      <c r="G40" s="25">
+      <c r="G40" s="24">
         <v>16.781549632752697</v>
       </c>
-      <c r="H40" s="25">
+      <c r="H40" s="24">
         <v>16.316953944920296</v>
       </c>
-      <c r="I40" s="25">
+      <c r="I40" s="24">
         <v>16.558768505166249</v>
       </c>
       <c r="J40" s="7"/>
       <c r="K40" s="7"/>
     </row>
-    <row r="41" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="23" t="s">
+    <row r="41" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C41" s="23">
+      <c r="C41" s="22">
         <v>2018</v>
       </c>
-      <c r="D41" s="24">
+      <c r="D41" s="23">
         <v>137.56186</v>
       </c>
-      <c r="E41" s="24">
+      <c r="E41" s="23">
         <v>133.2397</v>
       </c>
-      <c r="F41" s="24">
+      <c r="F41" s="23">
         <v>270.80155999999999</v>
       </c>
-      <c r="G41" s="25">
+      <c r="G41" s="24">
         <v>17.241570946074667</v>
       </c>
-      <c r="H41" s="25">
+      <c r="H41" s="24">
         <v>17.123951133140565</v>
       </c>
-      <c r="I41" s="25">
+      <c r="I41" s="24">
         <v>17.183498438855164</v>
       </c>
       <c r="J41" s="7"/>
       <c r="K41" s="7"/>
     </row>
-    <row r="42" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="23" t="s">
+    <row r="42" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C42" s="23">
+      <c r="C42" s="22">
         <v>2018</v>
       </c>
-      <c r="D42" s="24">
+      <c r="D42" s="23">
         <v>103.33179</v>
       </c>
-      <c r="E42" s="24">
+      <c r="E42" s="23">
         <v>114.24866</v>
       </c>
-      <c r="F42" s="24">
+      <c r="F42" s="23">
         <v>217.58044999999998</v>
       </c>
-      <c r="G42" s="25">
+      <c r="G42" s="24">
         <v>9.4200431598790022</v>
       </c>
-      <c r="H42" s="25">
+      <c r="H42" s="24">
         <v>10.257158554915771</v>
       </c>
-      <c r="I42" s="25">
+      <c r="I42" s="24">
         <v>9.8418019327751871</v>
       </c>
       <c r="J42" s="7"/>
       <c r="K42" s="7"/>
     </row>
-    <row r="43" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="23" t="s">
+    <row r="43" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C43" s="23">
+      <c r="C43" s="22">
         <v>2018</v>
       </c>
-      <c r="D43" s="24">
+      <c r="D43" s="23">
         <v>40.9163</v>
       </c>
-      <c r="E43" s="24">
+      <c r="E43" s="23">
         <v>52.757599999999996</v>
       </c>
-      <c r="F43" s="24">
+      <c r="F43" s="23">
         <v>93.673900000000003</v>
       </c>
-      <c r="G43" s="25">
+      <c r="G43" s="24">
         <v>5.6662749446833898</v>
       </c>
-      <c r="H43" s="25">
+      <c r="H43" s="24">
         <v>5.9866551205358798</v>
       </c>
-      <c r="I43" s="25">
+      <c r="I43" s="24">
         <v>5.8423657024713487</v>
       </c>
       <c r="J43" s="7"/>
       <c r="K43" s="7"/>
     </row>
-    <row r="44" spans="2:11" s="46" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="26" t="s">
+    <row r="44" spans="2:11" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C44" s="26">
+      <c r="C44" s="25">
         <v>2018</v>
       </c>
-      <c r="D44" s="28">
+      <c r="D44" s="27">
         <v>328.89071000000001</v>
       </c>
-      <c r="E44" s="28">
+      <c r="E44" s="27">
         <v>342.42012</v>
       </c>
-      <c r="F44" s="28">
+      <c r="F44" s="27">
         <v>671.31083000000001</v>
       </c>
-      <c r="G44" s="27">
+      <c r="G44" s="26">
         <v>11.351085731819232</v>
       </c>
-      <c r="H44" s="27">
+      <c r="H44" s="26">
         <v>11.294826375948235</v>
       </c>
-      <c r="I44" s="27">
+      <c r="I44" s="26">
         <v>11.322319285430122</v>
       </c>
       <c r="J44" s="13"/>
       <c r="K44" s="13"/>
     </row>
-    <row r="45" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="23" t="s">
+    <row r="45" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C45" s="23">
+      <c r="C45" s="22">
         <v>2017</v>
       </c>
-      <c r="D45" s="24">
+      <c r="D45" s="23">
         <v>53.054550000000006</v>
       </c>
-      <c r="E45" s="24">
+      <c r="E45" s="23">
         <v>42.716800000000006</v>
       </c>
-      <c r="F45" s="24">
+      <c r="F45" s="23">
         <v>95.771350000000012</v>
       </c>
-      <c r="G45" s="25">
+      <c r="G45" s="24">
         <v>18.439419952897143</v>
       </c>
-      <c r="H45" s="25">
+      <c r="H45" s="24">
         <v>16.111910732120929</v>
       </c>
-      <c r="I45" s="25">
+      <c r="I45" s="24">
         <v>17.323234279124218</v>
       </c>
       <c r="J45" s="7"/>
       <c r="K45" s="7"/>
     </row>
-    <row r="46" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="23" t="s">
+    <row r="46" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C46" s="23">
+      <c r="C46" s="22">
         <v>2017</v>
       </c>
-      <c r="D46" s="24">
+      <c r="D46" s="23">
         <v>144.42716000000001</v>
       </c>
-      <c r="E46" s="24">
+      <c r="E46" s="23">
         <v>137.24038000000002</v>
       </c>
-      <c r="F46" s="24">
+      <c r="F46" s="23">
         <v>281.66754000000003</v>
       </c>
-      <c r="G46" s="25">
+      <c r="G46" s="24">
         <v>17.820437552845892</v>
       </c>
-      <c r="H46" s="25">
+      <c r="H46" s="24">
         <v>17.486430438862701</v>
       </c>
-      <c r="I46" s="25">
+      <c r="I46" s="24">
         <v>17.656115885108061</v>
       </c>
       <c r="J46" s="7"/>
       <c r="K46" s="7"/>
     </row>
-    <row r="47" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="23" t="s">
+    <row r="47" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C47" s="23">
+      <c r="C47" s="22">
         <v>2017</v>
       </c>
-      <c r="D47" s="24">
+      <c r="D47" s="23">
         <v>110.92681</v>
       </c>
-      <c r="E47" s="24">
+      <c r="E47" s="23">
         <v>121.26992999999999</v>
       </c>
-      <c r="F47" s="24">
+      <c r="F47" s="23">
         <v>232.19673999999998</v>
       </c>
-      <c r="G47" s="25">
+      <c r="G47" s="24">
         <v>9.9407784816758706</v>
       </c>
-      <c r="H47" s="25">
+      <c r="H47" s="24">
         <v>10.773958080048111</v>
       </c>
-      <c r="I47" s="25">
+      <c r="I47" s="24">
         <v>10.359172452359093</v>
       </c>
       <c r="J47" s="7"/>
       <c r="K47" s="7"/>
     </row>
-    <row r="48" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="23" t="s">
+    <row r="48" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C48" s="23">
+      <c r="C48" s="22">
         <v>2017</v>
       </c>
-      <c r="D48" s="24">
+      <c r="D48" s="23">
         <v>41.625620000000005</v>
       </c>
-      <c r="E48" s="24">
+      <c r="E48" s="23">
         <v>50.156440000000003</v>
       </c>
-      <c r="F48" s="24">
+      <c r="F48" s="23">
         <v>91.782060000000001</v>
       </c>
-      <c r="G48" s="25">
+      <c r="G48" s="24">
         <v>5.9378318761718667</v>
       </c>
-      <c r="H48" s="25">
+      <c r="H48" s="24">
         <v>5.7947360652354281</v>
       </c>
-      <c r="I48" s="25">
+      <c r="I48" s="24">
         <v>5.8587697312925808</v>
       </c>
       <c r="J48" s="7"/>
       <c r="K48" s="7"/>
     </row>
-    <row r="49" spans="2:11" s="46" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="26" t="s">
+    <row r="49" spans="2:11" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C49" s="26">
+      <c r="C49" s="25">
         <v>2017</v>
       </c>
-      <c r="D49" s="28">
+      <c r="D49" s="27">
         <v>350.03414000000004</v>
       </c>
-      <c r="E49" s="28">
+      <c r="E49" s="27">
         <v>351.38353999999998</v>
       </c>
-      <c r="F49" s="28">
+      <c r="F49" s="27">
         <v>701.41768000000002</v>
       </c>
-      <c r="G49" s="27">
+      <c r="G49" s="26">
         <v>12.007694836952282</v>
       </c>
-      <c r="H49" s="27">
+      <c r="H49" s="26">
         <v>11.554486278898048</v>
       </c>
-      <c r="I49" s="27">
+      <c r="I49" s="26">
         <v>11.776296152756677</v>
       </c>
       <c r="J49" s="13"/>
       <c r="K49" s="13"/>
     </row>
-    <row r="50" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="23" t="s">
+    <row r="50" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C50" s="23">
+      <c r="C50" s="22">
         <v>2016</v>
       </c>
-      <c r="D50" s="24">
+      <c r="D50" s="23">
         <v>44.005269999999996</v>
       </c>
-      <c r="E50" s="24">
+      <c r="E50" s="23">
         <v>35.384910000000005</v>
       </c>
-      <c r="F50" s="24">
+      <c r="F50" s="23">
         <v>79.390180000000001</v>
       </c>
-      <c r="G50" s="25">
+      <c r="G50" s="24">
         <v>15.344135589650715</v>
       </c>
-      <c r="H50" s="25">
+      <c r="H50" s="24">
         <v>13.504670773150378</v>
       </c>
-      <c r="I50" s="25">
+      <c r="I50" s="24">
         <v>14.465912927318344</v>
       </c>
       <c r="J50" s="7"/>
       <c r="K50" s="7"/>
     </row>
-    <row r="51" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="23" t="s">
+    <row r="51" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C51" s="23">
+      <c r="C51" s="22">
         <v>2016</v>
       </c>
-      <c r="D51" s="24">
+      <c r="D51" s="23">
         <v>116.25483</v>
       </c>
-      <c r="E51" s="24">
+      <c r="E51" s="23">
         <v>111.55392000000001</v>
       </c>
-      <c r="F51" s="24">
+      <c r="F51" s="23">
         <v>227.80875</v>
       </c>
-      <c r="G51" s="25">
+      <c r="G51" s="24">
         <v>14.034230462259533</v>
       </c>
-      <c r="H51" s="25">
+      <c r="H51" s="24">
         <v>13.907508011371913</v>
       </c>
-      <c r="I51" s="25">
+      <c r="I51" s="24">
         <v>13.971889454167153</v>
       </c>
       <c r="J51" s="7"/>
       <c r="K51" s="7"/>
     </row>
-    <row r="52" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="23" t="s">
+    <row r="52" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C52" s="23">
+      <c r="C52" s="22">
         <v>2016</v>
       </c>
-      <c r="D52" s="24">
+      <c r="D52" s="23">
         <v>96.441009999999991</v>
       </c>
-      <c r="E52" s="24">
+      <c r="E52" s="23">
         <v>103.83453</v>
       </c>
-      <c r="F52" s="24">
+      <c r="F52" s="23">
         <v>200.27553999999998</v>
       </c>
-      <c r="G52" s="25">
+      <c r="G52" s="24">
         <v>8.5520009060556745</v>
       </c>
-      <c r="H52" s="25">
+      <c r="H52" s="24">
         <v>9.1208636156057601</v>
       </c>
-      <c r="I52" s="25">
+      <c r="I52" s="24">
         <v>8.8377787251492101</v>
       </c>
       <c r="J52" s="7"/>
       <c r="K52" s="7"/>
     </row>
-    <row r="53" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="23" t="s">
+    <row r="53" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C53" s="23">
+      <c r="C53" s="22">
         <v>2016</v>
       </c>
-      <c r="D53" s="24">
+      <c r="D53" s="23">
         <v>37.959120000000006</v>
       </c>
-      <c r="E53" s="24">
+      <c r="E53" s="23">
         <v>50.489629999999998</v>
       </c>
-      <c r="F53" s="24">
+      <c r="F53" s="23">
         <v>88.448750000000004</v>
       </c>
-      <c r="G53" s="25">
+      <c r="G53" s="24">
         <v>5.3032939010692299</v>
       </c>
-      <c r="H53" s="25">
+      <c r="H53" s="24">
         <v>5.4756996019379063</v>
       </c>
-      <c r="I53" s="25">
+      <c r="I53" s="24">
         <v>5.4003549093800007</v>
       </c>
       <c r="J53" s="7"/>
       <c r="K53" s="7"/>
     </row>
-    <row r="54" spans="2:11" s="46" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="26" t="s">
+    <row r="54" spans="2:11" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C54" s="26">
+      <c r="C54" s="25">
         <v>2016</v>
       </c>
-      <c r="D54" s="28">
+      <c r="D54" s="27">
         <v>294.66022999999996</v>
       </c>
-      <c r="E54" s="28">
+      <c r="E54" s="27">
         <v>301.26299</v>
       </c>
-      <c r="F54" s="28">
+      <c r="F54" s="27">
         <v>595.9232199999999</v>
       </c>
-      <c r="G54" s="27">
+      <c r="G54" s="26">
         <v>9.9593766853289623</v>
       </c>
-      <c r="H54" s="27">
+      <c r="H54" s="26">
         <v>9.6415614985949905</v>
       </c>
-      <c r="I54" s="27">
+      <c r="I54" s="26">
         <v>9.7961326204420125</v>
       </c>
       <c r="J54" s="13"/>
       <c r="K54" s="13"/>
     </row>
-    <row r="55" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="23" t="s">
+    <row r="55" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C55" s="23">
+      <c r="C55" s="22">
         <v>2015</v>
       </c>
-      <c r="D55" s="24">
+      <c r="D55" s="23">
         <v>39.851529999999997</v>
       </c>
-      <c r="E55" s="24">
+      <c r="E55" s="23">
         <v>36.345699999999994</v>
       </c>
-      <c r="F55" s="24">
+      <c r="F55" s="23">
         <v>76.19722999999999</v>
       </c>
-      <c r="G55" s="25">
+      <c r="G55" s="24">
         <v>14.319157564260006</v>
       </c>
-      <c r="H55" s="25">
+      <c r="H55" s="24">
         <v>14.011435995146496</v>
       </c>
-      <c r="I55" s="25">
+      <c r="I55" s="24">
         <v>14.17070740232322</v>
       </c>
       <c r="J55" s="7"/>
       <c r="K55" s="7"/>
     </row>
-    <row r="56" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="23" t="s">
+    <row r="56" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C56" s="23">
+      <c r="C56" s="22">
         <v>2015</v>
       </c>
-      <c r="D56" s="24">
+      <c r="D56" s="23">
         <v>106.21704</v>
       </c>
-      <c r="E56" s="24">
+      <c r="E56" s="23">
         <v>107.25866000000001</v>
       </c>
-      <c r="F56" s="24">
+      <c r="F56" s="23">
         <v>213.47570000000002</v>
       </c>
-      <c r="G56" s="25">
+      <c r="G56" s="24">
         <v>12.6894189278841</v>
       </c>
-      <c r="H56" s="25">
+      <c r="H56" s="24">
         <v>13.087934705056975</v>
       </c>
-      <c r="I56" s="25">
+      <c r="I56" s="24">
         <v>12.886568393274841</v>
       </c>
       <c r="J56" s="7"/>
       <c r="K56" s="7"/>
     </row>
-    <row r="57" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="23" t="s">
+    <row r="57" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C57" s="23">
+      <c r="C57" s="22">
         <v>2015</v>
       </c>
-      <c r="D57" s="24">
+      <c r="D57" s="23">
         <v>93.883449999999996</v>
       </c>
-      <c r="E57" s="24">
+      <c r="E57" s="23">
         <v>100.07469</v>
       </c>
-      <c r="F57" s="24">
+      <c r="F57" s="23">
         <v>193.95814000000001</v>
       </c>
-      <c r="G57" s="25">
+      <c r="G57" s="24">
         <v>8.4355978708858963</v>
       </c>
-      <c r="H57" s="25">
+      <c r="H57" s="24">
         <v>8.8227195460663896</v>
       </c>
-      <c r="I57" s="25">
+      <c r="I57" s="24">
         <v>8.6309968153336616</v>
       </c>
       <c r="J57" s="7"/>
       <c r="K57" s="7"/>
     </row>
-    <row r="58" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="23" t="s">
+    <row r="58" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C58" s="23">
+      <c r="C58" s="22">
         <v>2015</v>
       </c>
-      <c r="D58" s="24">
+      <c r="D58" s="23">
         <v>33.258040000000001</v>
       </c>
-      <c r="E58" s="24">
+      <c r="E58" s="23">
         <v>44.901480000000006</v>
       </c>
-      <c r="F58" s="24">
+      <c r="F58" s="23">
         <v>78.159520000000015</v>
       </c>
-      <c r="G58" s="25">
+      <c r="G58" s="24">
         <v>4.5546291419798681</v>
       </c>
-      <c r="H58" s="25">
+      <c r="H58" s="24">
         <v>4.8383188428484809</v>
       </c>
-      <c r="I58" s="25">
+      <c r="I58" s="24">
         <v>4.7133967323259851</v>
       </c>
       <c r="J58" s="7"/>
       <c r="K58" s="7"/>
     </row>
-    <row r="59" spans="2:11" s="46" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="26" t="s">
+    <row r="59" spans="2:11" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B59" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C59" s="26">
+      <c r="C59" s="25">
         <v>2015</v>
       </c>
-      <c r="D59" s="28">
+      <c r="D59" s="27">
         <v>273.21007000000003</v>
       </c>
-      <c r="E59" s="28">
+      <c r="E59" s="27">
         <v>288.58053999999998</v>
       </c>
-      <c r="F59" s="28">
+      <c r="F59" s="27">
         <v>561.79061000000002</v>
       </c>
-      <c r="G59" s="27">
+      <c r="G59" s="26">
         <v>9.2347250762275301</v>
       </c>
-      <c r="H59" s="27">
+      <c r="H59" s="26">
         <v>9.1868168565262902</v>
       </c>
-      <c r="I59" s="27">
+      <c r="I59" s="26">
         <v>9.2100533415925501</v>
       </c>
       <c r="J59" s="13"/>
       <c r="K59" s="13"/>
     </row>
-    <row r="60" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="23" t="s">
+    <row r="60" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C60" s="23">
+      <c r="C60" s="22">
         <v>2014</v>
       </c>
-      <c r="D60" s="24">
+      <c r="D60" s="23">
         <v>36.484699999999997</v>
       </c>
-      <c r="E60" s="24">
+      <c r="E60" s="23">
         <v>37.825530000000001</v>
       </c>
-      <c r="F60" s="24">
+      <c r="F60" s="23">
         <v>74.31022999999999</v>
       </c>
-      <c r="G60" s="25">
+      <c r="G60" s="24">
         <v>12.953367599713259</v>
       </c>
-      <c r="H60" s="25">
+      <c r="H60" s="24">
         <v>14.363902403236123</v>
       </c>
-      <c r="I60" s="25">
+      <c r="I60" s="24">
         <v>13.634921849717568</v>
       </c>
       <c r="J60" s="7"/>
       <c r="K60" s="7"/>
     </row>
-    <row r="61" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="23" t="s">
+    <row r="61" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C61" s="23">
+      <c r="C61" s="22">
         <v>2014</v>
       </c>
-      <c r="D61" s="24">
+      <c r="D61" s="23">
         <v>107.87508</v>
       </c>
-      <c r="E61" s="24">
+      <c r="E61" s="23">
         <v>109.11467999999999</v>
       </c>
-      <c r="F61" s="24">
+      <c r="F61" s="23">
         <v>216.98975999999999</v>
       </c>
-      <c r="G61" s="25">
+      <c r="G61" s="24">
         <v>12.740997185585199</v>
       </c>
-      <c r="H61" s="25">
+      <c r="H61" s="24">
         <v>13.151221654628973</v>
       </c>
-      <c r="I61" s="25">
+      <c r="I61" s="24">
         <v>12.944031274732581</v>
       </c>
       <c r="J61" s="7"/>
       <c r="K61" s="7"/>
     </row>
-    <row r="62" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="23" t="s">
+    <row r="62" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C62" s="23">
+      <c r="C62" s="22">
         <v>2014</v>
       </c>
-      <c r="D62" s="24">
+      <c r="D62" s="23">
         <v>93.629410000000007</v>
       </c>
-      <c r="E62" s="24">
+      <c r="E62" s="23">
         <v>99.10548</v>
       </c>
-      <c r="F62" s="24">
+      <c r="F62" s="23">
         <v>192.73489000000001</v>
       </c>
-      <c r="G62" s="25">
+      <c r="G62" s="24">
         <v>8.6036560503302084</v>
       </c>
-      <c r="H62" s="25">
+      <c r="H62" s="24">
         <v>9.0061574992793894</v>
       </c>
-      <c r="I62" s="25">
+      <c r="I62" s="24">
         <v>8.8060256085319679</v>
       </c>
       <c r="J62" s="7"/>
       <c r="K62" s="7"/>
     </row>
-    <row r="63" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="23" t="s">
+    <row r="63" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B63" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C63" s="23">
+      <c r="C63" s="22">
         <v>2014</v>
       </c>
-      <c r="D63" s="24">
+      <c r="D63" s="23">
         <v>35.691549999999999</v>
       </c>
-      <c r="E63" s="24">
+      <c r="E63" s="23">
         <v>45.269220000000004</v>
       </c>
-      <c r="F63" s="24">
+      <c r="F63" s="23">
         <v>80.960769999999997</v>
       </c>
-      <c r="G63" s="25">
+      <c r="G63" s="24">
         <v>4.9045488312654397</v>
       </c>
-      <c r="H63" s="25">
+      <c r="H63" s="24">
         <v>4.8487417153852039</v>
       </c>
-      <c r="I63" s="25">
+      <c r="I63" s="24">
         <v>4.8731869589002903</v>
       </c>
       <c r="J63" s="7"/>
       <c r="K63" s="7"/>
     </row>
-    <row r="64" spans="2:11" s="46" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="26" t="s">
+    <row r="64" spans="2:11" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B64" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C64" s="26">
+      <c r="C64" s="25">
         <v>2014</v>
       </c>
-      <c r="D64" s="28">
+      <c r="D64" s="27">
         <v>273.68074000000001</v>
       </c>
-      <c r="E64" s="28">
+      <c r="E64" s="27">
         <v>291.31491</v>
       </c>
-      <c r="F64" s="28">
+      <c r="F64" s="27">
         <v>564.99565000000007</v>
       </c>
-      <c r="G64" s="27">
+      <c r="G64" s="26">
         <v>9.2952305176292285</v>
       </c>
-      <c r="H64" s="27">
+      <c r="H64" s="26">
         <v>9.3158851418018607</v>
       </c>
-      <c r="I64" s="27">
+      <c r="I64" s="26">
         <v>9.3058687066249792</v>
       </c>
       <c r="J64" s="13"/>
       <c r="K64" s="13"/>
     </row>
-    <row r="65" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="23" t="s">
+    <row r="65" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C65" s="23">
+      <c r="C65" s="22">
         <v>2013</v>
       </c>
-      <c r="D65" s="24">
+      <c r="D65" s="23">
         <v>43.561419999999998</v>
       </c>
-      <c r="E65" s="24">
+      <c r="E65" s="23">
         <v>42.883629999999997</v>
       </c>
-      <c r="F65" s="24">
+      <c r="F65" s="23">
         <v>86.445049999999995</v>
       </c>
-      <c r="G65" s="25">
+      <c r="G65" s="24">
         <v>15.410178444827608</v>
       </c>
-      <c r="H65" s="25">
+      <c r="H65" s="24">
         <v>16.02359678447684</v>
       </c>
-      <c r="I65" s="25">
+      <c r="I65" s="24">
         <v>15.708498768106965</v>
       </c>
       <c r="J65" s="7"/>
       <c r="K65" s="7"/>
     </row>
-    <row r="66" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="23" t="s">
+    <row r="66" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C66" s="23">
+      <c r="C66" s="22">
         <v>2013</v>
       </c>
-      <c r="D66" s="24">
+      <c r="D66" s="23">
         <v>109.29798</v>
       </c>
-      <c r="E66" s="24">
+      <c r="E66" s="23">
         <v>106.54449000000001</v>
       </c>
-      <c r="F66" s="24">
+      <c r="F66" s="23">
         <v>215.84246999999999</v>
       </c>
-      <c r="G66" s="25">
+      <c r="G66" s="24">
         <v>12.743843612869247</v>
       </c>
-      <c r="H66" s="25">
+      <c r="H66" s="24">
         <v>12.6541880616247</v>
       </c>
-      <c r="I66" s="25">
+      <c r="I66" s="24">
         <v>12.699429478305122</v>
       </c>
       <c r="J66" s="7"/>
       <c r="K66" s="7"/>
     </row>
-    <row r="67" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="23" t="s">
+    <row r="67" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B67" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C67" s="23">
+      <c r="C67" s="22">
         <v>2013</v>
       </c>
-      <c r="D67" s="24">
+      <c r="D67" s="23">
         <v>95.905460000000005</v>
       </c>
-      <c r="E67" s="24">
+      <c r="E67" s="23">
         <v>100.40627000000001</v>
       </c>
-      <c r="F67" s="24">
+      <c r="F67" s="23">
         <v>196.31173000000001</v>
       </c>
-      <c r="G67" s="25">
+      <c r="G67" s="24">
         <v>8.8746589454064946</v>
       </c>
-      <c r="H67" s="25">
+      <c r="H67" s="24">
         <v>9.1661793558104687</v>
       </c>
-      <c r="I67" s="25">
+      <c r="I67" s="24">
         <v>9.0214060118099653</v>
       </c>
       <c r="J67" s="7"/>
       <c r="K67" s="7"/>
     </row>
-    <row r="68" spans="2:11" s="45" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="23" t="s">
+    <row r="68" spans="2:11" s="30" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B68" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C68" s="23">
+      <c r="C68" s="22">
         <v>2013</v>
       </c>
-      <c r="D68" s="24">
+      <c r="D68" s="23">
         <v>32.456249999999997</v>
       </c>
-      <c r="E68" s="24">
+      <c r="E68" s="23">
         <v>46.073459999999997</v>
       </c>
-      <c r="F68" s="24">
+      <c r="F68" s="23">
         <v>78.529709999999994</v>
       </c>
-      <c r="G68" s="25">
+      <c r="G68" s="24">
         <v>4.5794359596648713</v>
       </c>
-      <c r="H68" s="25">
+      <c r="H68" s="24">
         <v>4.9825264553691939</v>
       </c>
-      <c r="I68" s="25">
+      <c r="I68" s="24">
         <v>4.8076280791470127</v>
       </c>
       <c r="J68" s="7"/>
       <c r="K68" s="7"/>
     </row>
-    <row r="69" spans="2:11" s="46" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="26" t="s">
+    <row r="69" spans="2:11" s="31" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B69" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C69" s="26">
+      <c r="C69" s="25">
         <v>2013</v>
       </c>
-      <c r="D69" s="28">
+      <c r="D69" s="27">
         <v>281.22111000000001</v>
       </c>
-      <c r="E69" s="28">
+      <c r="E69" s="27">
         <v>295.90785999999997</v>
       </c>
-      <c r="F69" s="28">
+      <c r="F69" s="27">
         <v>577.12896999999998</v>
       </c>
-      <c r="G69" s="27">
+      <c r="G69" s="26">
         <v>9.5988478724704596</v>
       </c>
-      <c r="H69" s="27">
+      <c r="H69" s="26">
         <v>9.4548366194110027</v>
       </c>
-      <c r="I69" s="27">
+      <c r="I69" s="26">
         <v>9.5244660755135637</v>
       </c>
       <c r="J69" s="13"/>
       <c r="K69" s="13"/>
     </row>
-    <row r="70" spans="2:11" s="47" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="23" t="s">
+    <row r="70" spans="2:11" s="32" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B70" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C70" s="23">
+      <c r="C70" s="22">
         <v>2012</v>
       </c>
-      <c r="D70" s="24">
+      <c r="D70" s="23">
         <v>46.041519999999998</v>
       </c>
-      <c r="E70" s="24">
+      <c r="E70" s="23">
         <v>39.716989999999996</v>
       </c>
-      <c r="F70" s="24">
+      <c r="F70" s="23">
         <v>85.758510000000001</v>
       </c>
-      <c r="G70" s="25">
+      <c r="G70" s="24">
         <v>15.829973271126754</v>
       </c>
-      <c r="H70" s="25">
+      <c r="H70" s="24">
         <v>14.790328045812377</v>
       </c>
-      <c r="I70" s="25">
+      <c r="I70" s="24">
         <v>15.330889096180472</v>
       </c>
       <c r="J70" s="6"/>
       <c r="K70" s="6"/>
     </row>
-    <row r="71" spans="2:11" s="47" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="23" t="s">
+    <row r="71" spans="2:11" s="32" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B71" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C71" s="23">
+      <c r="C71" s="22">
         <v>2012</v>
       </c>
-      <c r="D71" s="24">
+      <c r="D71" s="23">
         <v>101.17434</v>
       </c>
-      <c r="E71" s="24">
+      <c r="E71" s="23">
         <v>105.36062</v>
       </c>
-      <c r="F71" s="24">
+      <c r="F71" s="23">
         <v>206.53496000000001</v>
       </c>
-      <c r="G71" s="25">
+      <c r="G71" s="24">
         <v>11.689085286571911</v>
       </c>
-      <c r="H71" s="25">
+      <c r="H71" s="24">
         <v>12.196344808456583</v>
       </c>
-      <c r="I71" s="25">
+      <c r="I71" s="24">
         <v>11.942469406982308</v>
       </c>
       <c r="J71" s="6"/>
       <c r="K71" s="6"/>
     </row>
-    <row r="72" spans="2:11" s="47" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="23" t="s">
+    <row r="72" spans="2:11" s="32" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B72" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C72" s="23">
+      <c r="C72" s="22">
         <v>2012</v>
       </c>
-      <c r="D72" s="24">
+      <c r="D72" s="23">
         <v>93.794139999999999</v>
       </c>
-      <c r="E72" s="24">
+      <c r="E72" s="23">
         <v>98.775850000000005</v>
       </c>
-      <c r="F72" s="24">
+      <c r="F72" s="23">
         <v>192.56999000000002</v>
       </c>
-      <c r="G72" s="25">
+      <c r="G72" s="24">
         <v>8.6753229662419784</v>
       </c>
-      <c r="H72" s="25">
+      <c r="H72" s="24">
         <v>9.1959978691350237</v>
       </c>
-      <c r="I72" s="25">
+      <c r="I72" s="24">
         <v>8.9348097603427039</v>
       </c>
       <c r="J72" s="6"/>
       <c r="K72" s="6"/>
     </row>
-    <row r="73" spans="2:11" s="47" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="23" t="s">
+    <row r="73" spans="2:11" s="32" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B73" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C73" s="23">
+      <c r="C73" s="22">
         <v>2012</v>
       </c>
-      <c r="D73" s="24">
+      <c r="D73" s="23">
         <v>30.689880000000002</v>
       </c>
-      <c r="E73" s="24">
+      <c r="E73" s="23">
         <v>45.083239999999996</v>
       </c>
-      <c r="F73" s="24">
+      <c r="F73" s="23">
         <v>75.773120000000006</v>
       </c>
-      <c r="G73" s="25">
+      <c r="G73" s="24">
         <v>4.4626134481040376</v>
       </c>
-      <c r="H73" s="25">
+      <c r="H73" s="24">
         <v>4.8949431553146123</v>
       </c>
-      <c r="I73" s="25">
+      <c r="I73" s="24">
         <v>4.7101276080597216</v>
       </c>
       <c r="J73" s="6"/>
       <c r="K73" s="6"/>
     </row>
-    <row r="74" spans="2:11" s="48" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="26" t="s">
+    <row r="74" spans="2:11" s="33" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B74" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C74" s="26">
+      <c r="C74" s="25">
         <v>2012</v>
       </c>
-      <c r="D74" s="28">
+      <c r="D74" s="27">
         <v>271.69988000000001</v>
       </c>
-      <c r="E74" s="28">
+      <c r="E74" s="27">
         <v>288.93670000000003</v>
       </c>
-      <c r="F74" s="28">
+      <c r="F74" s="27">
         <v>560.63658000000009</v>
       </c>
-      <c r="G74" s="27">
+      <c r="G74" s="26">
         <v>9.2880375902806556</v>
       </c>
-      <c r="H74" s="27">
+      <c r="H74" s="26">
         <v>9.2384700720590036</v>
       </c>
-      <c r="I74" s="27">
+      <c r="I74" s="26">
         <v>9.2624256117437511</v>
       </c>
       <c r="J74" s="14"/>
       <c r="K74" s="14"/>
     </row>
-    <row r="75" spans="2:11" s="47" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="23" t="s">
+    <row r="75" spans="2:11" s="32" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B75" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C75" s="23">
+      <c r="C75" s="22">
         <v>2011</v>
       </c>
-      <c r="D75" s="24">
+      <c r="D75" s="23">
         <v>49.395949999999999</v>
       </c>
-      <c r="E75" s="24">
+      <c r="E75" s="23">
         <v>43.41377</v>
       </c>
-      <c r="F75" s="24">
+      <c r="F75" s="23">
         <v>92.809719999999999</v>
       </c>
-      <c r="G75" s="25">
+      <c r="G75" s="24">
         <v>16.374816331764272</v>
       </c>
-      <c r="H75" s="25">
+      <c r="H75" s="24">
         <v>15.398537063837336</v>
       </c>
-      <c r="I75" s="25">
+      <c r="I75" s="24">
         <v>15.903174342120485</v>
       </c>
       <c r="J75" s="6"/>
       <c r="K75" s="6"/>
     </row>
-    <row r="76" spans="2:11" s="47" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="23" t="s">
+    <row r="76" spans="2:11" s="32" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="C76" s="23">
+      <c r="C76" s="22">
         <v>2011</v>
       </c>
-      <c r="D76" s="24">
+      <c r="D76" s="23">
         <v>101.92383</v>
       </c>
-      <c r="E76" s="24">
+      <c r="E76" s="23">
         <v>104.17531</v>
       </c>
-      <c r="F76" s="24">
+      <c r="F76" s="23">
         <v>206.09913999999998</v>
       </c>
-      <c r="G76" s="25">
+      <c r="G76" s="24">
         <v>11.536175825357917</v>
       </c>
-      <c r="H76" s="25">
+      <c r="H76" s="24">
         <v>11.835846259409939</v>
       </c>
-      <c r="I76" s="25">
+      <c r="I76" s="24">
         <v>11.685726689953926</v>
       </c>
       <c r="J76" s="6"/>
       <c r="K76" s="6"/>
     </row>
-    <row r="77" spans="2:11" s="49" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="23" t="s">
+    <row r="77" spans="2:11" s="34" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B77" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C77" s="23">
+      <c r="C77" s="22">
         <v>2011</v>
       </c>
-      <c r="D77" s="24">
+      <c r="D77" s="23">
         <v>86.011289999999988</v>
       </c>
-      <c r="E77" s="24">
+      <c r="E77" s="23">
         <v>96.004519999999999</v>
       </c>
-      <c r="F77" s="24">
+      <c r="F77" s="23">
         <v>182.01580999999999</v>
       </c>
-      <c r="G77" s="25">
+      <c r="G77" s="24">
         <v>8.1601077357144955</v>
       </c>
-      <c r="H77" s="25">
+      <c r="H77" s="24">
         <v>9.089852014992287</v>
       </c>
-      <c r="I77" s="25">
+      <c r="I77" s="24">
         <v>8.6254483386351062</v>
       </c>
       <c r="J77" s="7"/>
       <c r="K77" s="6"/>
     </row>
-    <row r="78" spans="2:11" s="49" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="23" t="s">
+    <row r="78" spans="2:11" s="34" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B78" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C78" s="23">
+      <c r="C78" s="22">
         <v>2011</v>
       </c>
-      <c r="D78" s="24">
+      <c r="D78" s="23">
         <v>31.317979999999999</v>
       </c>
-      <c r="E78" s="24">
+      <c r="E78" s="23">
         <v>42.319459999999999</v>
       </c>
-      <c r="F78" s="24">
+      <c r="F78" s="23">
         <v>73.637439999999998</v>
       </c>
-      <c r="G78" s="25">
+      <c r="G78" s="24">
         <v>4.5506122254154278</v>
       </c>
-      <c r="H78" s="25">
+      <c r="H78" s="24">
         <v>4.6011067847012033</v>
       </c>
-      <c r="I78" s="25">
+      <c r="I78" s="24">
         <v>4.5794951597736251</v>
       </c>
       <c r="J78" s="7"/>
       <c r="K78" s="6"/>
     </row>
-    <row r="79" spans="2:11" s="49" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="26" t="s">
+    <row r="79" spans="2:11" s="34" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B79" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="C79" s="26">
+      <c r="C79" s="25">
         <v>2011</v>
       </c>
-      <c r="D79" s="28">
+      <c r="D79" s="27">
         <v>268.64904999999999</v>
       </c>
-      <c r="E79" s="28">
+      <c r="E79" s="27">
         <v>285.91305999999997</v>
       </c>
-      <c r="F79" s="28">
+      <c r="F79" s="27">
         <v>554.56210999999996</v>
       </c>
-      <c r="G79" s="27">
+      <c r="G79" s="26">
         <v>9.1769477795528598</v>
       </c>
-      <c r="H79" s="27">
+      <c r="H79" s="26">
         <v>9.1111938031645465</v>
       </c>
-      <c r="I79" s="27">
+      <c r="I79" s="26">
         <v>9.142929222004609</v>
       </c>
       <c r="J79" s="7"/>
@@ -2937,7 +2950,7 @@
       <c r="I80" s="18"/>
       <c r="J80" s="15"/>
     </row>
-    <row r="81" spans="2:10" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:13" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="19"/>
       <c r="C81" s="20"/>
       <c r="D81" s="20"/>
@@ -2948,90 +2961,182 @@
       <c r="I81" s="20"/>
       <c r="J81" s="15"/>
     </row>
-    <row r="82" spans="2:10" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="51" t="s">
+    <row r="82" spans="2:13" s="8" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="C82" s="50"/>
+      <c r="D82" s="50"/>
+      <c r="E82" s="50"/>
+      <c r="F82" s="50"/>
+      <c r="G82" s="50"/>
+      <c r="H82" s="50"/>
+      <c r="I82" s="50"/>
+      <c r="J82" s="50"/>
+      <c r="K82" s="50"/>
+      <c r="L82" s="50"/>
+      <c r="M82" s="50"/>
+    </row>
+    <row r="83" spans="2:13" s="8" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B83" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="C83" s="50"/>
+      <c r="D83" s="50"/>
+      <c r="E83" s="50"/>
+      <c r="F83" s="50"/>
+      <c r="G83" s="50"/>
+      <c r="H83" s="50"/>
+      <c r="I83" s="50"/>
+      <c r="J83" s="50"/>
+      <c r="K83" s="50"/>
+      <c r="L83" s="50"/>
+      <c r="M83" s="50"/>
+    </row>
+    <row r="84" spans="2:13" s="8" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="C84" s="50"/>
+      <c r="D84" s="50"/>
+      <c r="E84" s="50"/>
+      <c r="F84" s="50"/>
+      <c r="G84" s="50"/>
+      <c r="H84" s="50"/>
+      <c r="I84" s="50"/>
+      <c r="J84" s="50"/>
+      <c r="K84" s="50"/>
+      <c r="L84" s="50"/>
+      <c r="M84" s="50"/>
+    </row>
+    <row r="85" spans="2:13" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B85" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="C82" s="15"/>
-      <c r="D82" s="15"/>
-      <c r="E82" s="15"/>
-      <c r="F82" s="15"/>
-      <c r="G82" s="15"/>
-      <c r="H82" s="15"/>
-      <c r="I82" s="15"/>
-    </row>
-    <row r="83" spans="2:10" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="51" t="s">
+      <c r="C85" s="52"/>
+      <c r="D85" s="52"/>
+      <c r="E85" s="52"/>
+      <c r="F85" s="52"/>
+      <c r="G85" s="52"/>
+      <c r="H85" s="52"/>
+      <c r="I85" s="52"/>
+      <c r="J85" s="52"/>
+      <c r="K85" s="52"/>
+      <c r="L85" s="52"/>
+      <c r="M85" s="52"/>
+    </row>
+    <row r="86" spans="2:13" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B86" s="51"/>
+      <c r="C86" s="52"/>
+      <c r="D86" s="52"/>
+      <c r="E86" s="52"/>
+      <c r="F86" s="52"/>
+      <c r="G86" s="52"/>
+      <c r="H86" s="52"/>
+      <c r="I86" s="52"/>
+      <c r="J86" s="52"/>
+      <c r="K86" s="52"/>
+      <c r="L86" s="52"/>
+      <c r="M86" s="52"/>
+    </row>
+    <row r="87" spans="2:13" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B87" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="C83" s="15"/>
-      <c r="D83" s="15"/>
-      <c r="E83" s="15"/>
-      <c r="F83" s="15"/>
-      <c r="G83" s="15"/>
-      <c r="H83" s="15"/>
-      <c r="I83" s="15"/>
-    </row>
-    <row r="84" spans="2:10" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B84" s="21" t="s">
+      <c r="C87" s="52"/>
+      <c r="D87" s="52"/>
+      <c r="E87" s="52"/>
+      <c r="F87" s="52"/>
+      <c r="G87" s="52"/>
+      <c r="H87" s="52"/>
+      <c r="I87" s="52"/>
+      <c r="J87" s="52"/>
+      <c r="K87" s="52"/>
+      <c r="L87" s="52"/>
+      <c r="M87" s="52"/>
+    </row>
+    <row r="88" spans="2:13" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B88" s="52"/>
+      <c r="C88" s="52"/>
+      <c r="D88" s="52"/>
+      <c r="E88" s="52"/>
+      <c r="F88" s="52"/>
+      <c r="G88" s="52"/>
+      <c r="H88" s="52"/>
+      <c r="I88" s="52"/>
+      <c r="J88" s="52"/>
+      <c r="K88" s="52"/>
+      <c r="L88" s="52"/>
+      <c r="M88" s="52"/>
+    </row>
+    <row r="89" spans="2:13" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B89" s="54" t="s">
+        <v>23</v>
+      </c>
+      <c r="C89" s="52"/>
+      <c r="D89" s="52"/>
+      <c r="E89" s="52"/>
+      <c r="F89" s="52"/>
+      <c r="G89" s="52"/>
+      <c r="H89" s="52"/>
+      <c r="I89" s="52"/>
+      <c r="J89" s="52"/>
+      <c r="K89" s="52"/>
+      <c r="L89" s="52"/>
+      <c r="M89" s="52"/>
+    </row>
+    <row r="90" spans="2:13" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B90" s="54" t="s">
+        <v>24</v>
+      </c>
+      <c r="C90" s="52"/>
+      <c r="D90" s="52"/>
+      <c r="E90" s="52"/>
+      <c r="F90" s="52"/>
+      <c r="G90" s="52"/>
+      <c r="H90" s="52"/>
+      <c r="I90" s="52"/>
+      <c r="J90" s="52"/>
+      <c r="K90" s="52"/>
+      <c r="L90" s="52"/>
+      <c r="M90" s="52"/>
+    </row>
+    <row r="91" spans="2:13" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B91" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="C84" s="7"/>
-      <c r="D84" s="7"/>
-      <c r="E84" s="7"/>
-      <c r="F84" s="7"/>
-      <c r="G84" s="7"/>
-      <c r="H84" s="7"/>
-      <c r="I84" s="7"/>
-    </row>
-    <row r="85" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25">
-      <c r="B85" s="15"/>
-      <c r="C85" s="15"/>
-      <c r="D85" s="15"/>
-      <c r="E85" s="15"/>
-      <c r="F85" s="15"/>
-      <c r="G85" s="15"/>
-      <c r="H85" s="15"/>
-      <c r="I85" s="15"/>
-    </row>
-    <row r="86" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25">
-      <c r="B86" s="7" t="s">
+      <c r="C91" s="52"/>
+      <c r="D91" s="52"/>
+      <c r="E91" s="52"/>
+      <c r="F91" s="52"/>
+      <c r="G91" s="52"/>
+      <c r="H91" s="52"/>
+      <c r="I91" s="52"/>
+      <c r="J91" s="52"/>
+      <c r="K91" s="52"/>
+      <c r="L91" s="52"/>
+      <c r="M91" s="52"/>
+    </row>
+    <row r="92" spans="2:13" s="8" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B92" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="C86" s="7"/>
-      <c r="D86" s="15"/>
-      <c r="E86" s="15"/>
-      <c r="F86" s="15"/>
-      <c r="G86" s="15"/>
-      <c r="H86" s="15"/>
-      <c r="I86" s="15"/>
-    </row>
-    <row r="87" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25">
-      <c r="B88" s="8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="89" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25">
-      <c r="B89" s="8" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="90" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25">
-      <c r="B90" s="8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="91" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25">
-      <c r="B91" s="8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="92" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="2:10" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
+      <c r="C92" s="52"/>
+      <c r="D92" s="52"/>
+      <c r="E92" s="52"/>
+      <c r="F92" s="52"/>
+      <c r="G92" s="52"/>
+      <c r="H92" s="52"/>
+      <c r="I92" s="52"/>
+      <c r="J92" s="52"/>
+      <c r="K92" s="52"/>
+      <c r="L92" s="52"/>
+      <c r="M92" s="52"/>
+    </row>
+    <row r="93" spans="2:13" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="2:13" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="2:13" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="2:13" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
     <row r="97" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
     <row r="98" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
     <row r="99" s="8" customFormat="1" ht="8.25" x14ac:dyDescent="0.25"/>
@@ -3217,7 +3322,10 @@
       <c r="I215" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
+    <mergeCell ref="B82:M82"/>
+    <mergeCell ref="B83:M83"/>
+    <mergeCell ref="B84:M84"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:C8"/>
     <mergeCell ref="D6:F6"/>
@@ -3226,8 +3334,8 @@
     <mergeCell ref="G8:I8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B91" r:id="rId1" xr:uid="{1C4C458E-2252-4458-B9C9-92C2BDC9901A}"/>
-    <hyperlink ref="B84" r:id="rId2" xr:uid="{44B0D61C-0819-4B8E-B245-71AADB05D95D}"/>
+    <hyperlink ref="B85" r:id="rId1" xr:uid="{DA9A39D6-7B7E-4BC9-A0F0-B092D2C551A3}"/>
+    <hyperlink ref="B92" r:id="rId2" xr:uid="{2DE976D6-87DA-4A81-914A-6FAD99A74485}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>

</xml_diff>